<commit_message>
Added data driven framework
</commit_message>
<xml_diff>
--- a/ParaBank/testdata/ParaBankData1.xlsx
+++ b/ParaBank/testdata/ParaBankData1.xlsx
@@ -5,17 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PRATHA\Desktop\eclipse_new\ParaBank\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PRATHA\git\Para-Bank-Automation-\ParaBank\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1415986B-02D6-4517-8DB2-91E623DA0A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7389F54A-FA47-4D89-856D-A9DFB17B052B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RegistrationData" sheetId="1" r:id="rId1"/>
+    <sheet name="LoginData" sheetId="2" r:id="rId2"/>
+    <sheet name="TransferData" sheetId="3" r:id="rId3"/>
+    <sheet name="BillPayData" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,13 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
   <si>
     <t>username</t>
   </si>
@@ -39,46 +36,73 @@
     <t>password</t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>user1780764750941</t>
-  </si>
-  <si>
     <t>Test123</t>
   </si>
   <si>
-    <t>user1780766950178</t>
-  </si>
-  <si>
-    <t>user1780821596912</t>
-  </si>
-  <si>
-    <t>user1780822467776</t>
-  </si>
-  <si>
-    <t>user1780823503242</t>
-  </si>
-  <si>
-    <t>user1780825919406</t>
-  </si>
-  <si>
-    <t>user1780826836256</t>
-  </si>
-  <si>
-    <t>user1780847898065</t>
-  </si>
-  <si>
-    <t>user1781291186210</t>
-  </si>
-  <si>
-    <t>user1781303190332</t>
-  </si>
-  <si>
-    <t>user1781303319894</t>
-  </si>
-  <si>
-    <t>user1781325927586</t>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>zipCode</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>ssn</t>
+  </si>
+  <si>
+    <t>Pratha</t>
+  </si>
+  <si>
+    <t>Khare</t>
+  </si>
+  <si>
+    <t>Jyendra Nagar</t>
+  </si>
+  <si>
+    <t>Mahoba</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>user1781</t>
+  </si>
+  <si>
+    <t>transferAmount</t>
+  </si>
+  <si>
+    <t>payeeName</t>
+  </si>
+  <si>
+    <t>account</t>
+  </si>
+  <si>
+    <t>verifyAccount</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>Electricity Board</t>
+  </si>
+  <si>
+    <t>user1781446128110</t>
+  </si>
+  <si>
+    <t>user1781447974065</t>
   </si>
 </sst>
 </file>
@@ -411,10 +435,85 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="14.77734375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2">
+        <v>210421</v>
+      </c>
+      <c r="G2" s="2">
+        <v>7080852802</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1234</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA1F4E61-E2C4-41BE-88B9-E6948D875C42}">
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -422,20 +521,100 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2100888-0D1F-43E8-B63C-0B7044B9F632}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF9912FD-B07A-4F64-BD6B-089D91D5AE2A}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2">
+        <v>210421</v>
+      </c>
+      <c r="F2" s="2">
+        <v>7080852802</v>
+      </c>
+      <c r="G2" s="2">
+        <v>12345</v>
+      </c>
+      <c r="H2" s="2">
+        <v>12345</v>
+      </c>
+      <c r="I2" s="2">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>